<commit_message>
this is my second commit
</commit_message>
<xml_diff>
--- a/bharat.xlsx
+++ b/bharat.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t xml:space="preserve">bharat </t>
   </si>
@@ -28,6 +28,9 @@
   </si>
   <si>
     <t>PRISHA PUROHIT</t>
+  </si>
+  <si>
+    <t>this sis sc lknlkv</t>
   </si>
 </sst>
 </file>
@@ -382,6 +385,11 @@
         <v>2</v>
       </c>
     </row>
+    <row r="13" spans="6:11" x14ac:dyDescent="0.3">
+      <c r="H13" t="s">
+        <v>4</v>
+      </c>
+    </row>
     <row r="17" spans="9:9" x14ac:dyDescent="0.3">
       <c r="I17" t="s">
         <v>3</v>

</xml_diff>